<commit_message>
Update ECON 3300 materials
</commit_message>
<xml_diff>
--- a/data/project/MetroRide_Student_Data/MetroRide_Data_Dictionary.xlsx
+++ b/data/project/MetroRide_Student_Data/MetroRide_Data_Dictionary.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="1" r:id="Rd8503be2a93f4381"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="1" r:id="Ra700579d4b83480e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -969,16 +969,16 @@
         <x:v>rides.csv</x:v>
       </x:c>
       <x:c r="B39" s="13" t="str">
-        <x:v>discount_amount</x:v>
+        <x:v>campaign_id</x:v>
       </x:c>
       <x:c r="C39" s="13" t="str">
-        <x:v>double</x:v>
+        <x:v>character</x:v>
       </x:c>
       <x:c r="D39" s="13" t="str">
-        <x:v>Ordinary ride discount applied</x:v>
+        <x:v>Campaign linked to a request during its 30-day follow-up window</x:v>
       </x:c>
       <x:c r="E39" s="13" t="str">
-        <x:v>USD</x:v>
+        <x:v>WINBACK_2025_06; blank outside window</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -986,16 +986,16 @@
         <x:v>rides.csv</x:v>
       </x:c>
       <x:c r="B40" s="13" t="str">
-        <x:v>amount_paid</x:v>
+        <x:v>campaign_treatment</x:v>
       </x:c>
       <x:c r="C40" s="13" t="str">
-        <x:v>double</x:v>
+        <x:v>character</x:v>
       </x:c>
       <x:c r="D40" s="13" t="str">
-        <x:v>Total amount paid for completed request including Priority fee</x:v>
+        <x:v>Customer's randomly assigned campaign condition</x:v>
       </x:c>
       <x:c r="E40" s="13" t="str">
-        <x:v>USD; zero if not completed</x:v>
+        <x:v>Five conditions; blank outside window</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -1003,13 +1003,13 @@
         <x:v>rides.csv</x:v>
       </x:c>
       <x:c r="B41" s="13" t="str">
-        <x:v>completed</x:v>
+        <x:v>campaign_offer_applied</x:v>
       </x:c>
       <x:c r="C41" s="13" t="str">
         <x:v>integer</x:v>
       </x:c>
       <x:c r="D41" s="13" t="str">
-        <x:v>Whether requested ride was completed</x:v>
+        <x:v>Whether the assigned financial offer was applied to this completed ride</x:v>
       </x:c>
       <x:c r="E41" s="13" t="str">
         <x:v>1=yes; 0=no</x:v>
@@ -1020,16 +1020,16 @@
         <x:v>rides.csv</x:v>
       </x:c>
       <x:c r="B42" s="13" t="str">
-        <x:v>customer_cancelled</x:v>
+        <x:v>discount_amount</x:v>
       </x:c>
       <x:c r="C42" s="13" t="str">
-        <x:v>integer</x:v>
+        <x:v>double</x:v>
       </x:c>
       <x:c r="D42" s="13" t="str">
-        <x:v>Whether customer cancelled the request</x:v>
+        <x:v>Campaign discount applied to this completed ride</x:v>
       </x:c>
       <x:c r="E42" s="13" t="str">
-        <x:v>1=yes; 0=no</x:v>
+        <x:v>USD; zero unless $5 off or 20% off was redeemed</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -1037,16 +1037,16 @@
         <x:v>rides.csv</x:v>
       </x:c>
       <x:c r="B43" s="13" t="str">
-        <x:v>driver_cancelled</x:v>
+        <x:v>ride_credit_earned</x:v>
       </x:c>
       <x:c r="C43" s="13" t="str">
-        <x:v>integer</x:v>
+        <x:v>double</x:v>
       </x:c>
       <x:c r="D43" s="13" t="str">
-        <x:v>Whether driver cancelled the request</x:v>
+        <x:v>Account credit earned after this completed ride</x:v>
       </x:c>
       <x:c r="E43" s="13" t="str">
-        <x:v>1=yes; 0=no</x:v>
+        <x:v>USD; zero unless $5 ride credit was redeemed</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -1054,16 +1054,16 @@
         <x:v>rides.csv</x:v>
       </x:c>
       <x:c r="B44" s="13" t="str">
-        <x:v>actual_wait_min</x:v>
+        <x:v>amount_paid</x:v>
       </x:c>
       <x:c r="C44" s="13" t="str">
         <x:v>double</x:v>
       </x:c>
       <x:c r="D44" s="13" t="str">
-        <x:v>Observed time until pickup or cancellation</x:v>
+        <x:v>Total amount paid for completed request including Priority fee</x:v>
       </x:c>
       <x:c r="E44" s="13" t="str">
-        <x:v>Minutes</x:v>
+        <x:v>USD; zero if not completed</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -1071,16 +1071,16 @@
         <x:v>rides.csv</x:v>
       </x:c>
       <x:c r="B45" s="13" t="str">
-        <x:v>actual_duration_min</x:v>
+        <x:v>completed</x:v>
       </x:c>
       <x:c r="C45" s="13" t="str">
-        <x:v>double</x:v>
+        <x:v>integer</x:v>
       </x:c>
       <x:c r="D45" s="13" t="str">
-        <x:v>Observed trip duration or last expected duration if cancelled</x:v>
+        <x:v>Whether requested ride was completed</x:v>
       </x:c>
       <x:c r="E45" s="13" t="str">
-        <x:v>Minutes</x:v>
+        <x:v>1=yes; 0=no</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -1088,16 +1088,16 @@
         <x:v>rides.csv</x:v>
       </x:c>
       <x:c r="B46" s="13" t="str">
-        <x:v>driver_id</x:v>
+        <x:v>customer_cancelled</x:v>
       </x:c>
       <x:c r="C46" s="13" t="str">
-        <x:v>character</x:v>
+        <x:v>integer</x:v>
       </x:c>
       <x:c r="D46" s="13" t="str">
-        <x:v>Fictional driver identifier</x:v>
+        <x:v>Whether customer cancelled the request</x:v>
       </x:c>
       <x:c r="E46" s="13" t="str">
-        <x:v>D####</x:v>
+        <x:v>1=yes; 0=no</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -1105,16 +1105,16 @@
         <x:v>rides.csv</x:v>
       </x:c>
       <x:c r="B47" s="13" t="str">
-        <x:v>driver_experience_months</x:v>
+        <x:v>driver_cancelled</x:v>
       </x:c>
       <x:c r="C47" s="13" t="str">
         <x:v>integer</x:v>
       </x:c>
       <x:c r="D47" s="13" t="str">
-        <x:v>Driver's experience with MetroRide before request</x:v>
+        <x:v>Whether driver cancelled the request</x:v>
       </x:c>
       <x:c r="E47" s="13" t="str">
-        <x:v>Months</x:v>
+        <x:v>1=yes; 0=no</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -1122,16 +1122,16 @@
         <x:v>rides.csv</x:v>
       </x:c>
       <x:c r="B48" s="13" t="str">
-        <x:v>driver_rating_before_ride</x:v>
+        <x:v>actual_wait_min</x:v>
       </x:c>
       <x:c r="C48" s="13" t="str">
         <x:v>double</x:v>
       </x:c>
       <x:c r="D48" s="13" t="str">
-        <x:v>Driver's average rating before request</x:v>
+        <x:v>Observed time until pickup or cancellation</x:v>
       </x:c>
       <x:c r="E48" s="13" t="str">
-        <x:v>1-5</x:v>
+        <x:v>Minutes</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -1139,16 +1139,16 @@
         <x:v>rides.csv</x:v>
       </x:c>
       <x:c r="B49" s="13" t="str">
-        <x:v>vehicle_quality</x:v>
+        <x:v>actual_duration_min</x:v>
       </x:c>
       <x:c r="C49" s="13" t="str">
-        <x:v>character</x:v>
+        <x:v>double</x:v>
       </x:c>
       <x:c r="D49" s="13" t="str">
-        <x:v>MetroRide vehicle category</x:v>
+        <x:v>Observed trip duration or last expected duration if cancelled</x:v>
       </x:c>
       <x:c r="E49" s="13" t="str">
-        <x:v>Standard; Comfort; Premium</x:v>
+        <x:v>Minutes</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -1156,16 +1156,16 @@
         <x:v>rides.csv</x:v>
       </x:c>
       <x:c r="B50" s="13" t="str">
-        <x:v>customer_rating</x:v>
+        <x:v>driver_id</x:v>
       </x:c>
       <x:c r="C50" s="13" t="str">
-        <x:v>integer</x:v>
+        <x:v>character</x:v>
       </x:c>
       <x:c r="D50" s="13" t="str">
-        <x:v>Rating submitted after completed ride</x:v>
+        <x:v>Fictional driver identifier</x:v>
       </x:c>
       <x:c r="E50" s="13" t="str">
-        <x:v>1-5; blank if no rating</x:v>
+        <x:v>D####</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -1173,84 +1173,84 @@
         <x:v>rides.csv</x:v>
       </x:c>
       <x:c r="B51" s="13" t="str">
-        <x:v>complaint</x:v>
+        <x:v>driver_experience_months</x:v>
       </x:c>
       <x:c r="C51" s="13" t="str">
         <x:v>integer</x:v>
       </x:c>
       <x:c r="D51" s="13" t="str">
-        <x:v>Whether customer filed a complaint about request</x:v>
+        <x:v>Driver's experience with MetroRide before request</x:v>
       </x:c>
       <x:c r="E51" s="13" t="str">
-        <x:v>1=yes; 0=no</x:v>
+        <x:v>Months</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="13" t="str">
-        <x:v>marketing_experiment.csv</x:v>
+        <x:v>rides.csv</x:v>
       </x:c>
       <x:c r="B52" s="13" t="str">
-        <x:v>campaign_id</x:v>
+        <x:v>driver_rating_before_ride</x:v>
       </x:c>
       <x:c r="C52" s="13" t="str">
-        <x:v>character</x:v>
+        <x:v>double</x:v>
       </x:c>
       <x:c r="D52" s="13" t="str">
-        <x:v>Campaign identifier</x:v>
+        <x:v>Driver's average rating before request</x:v>
       </x:c>
       <x:c r="E52" s="13" t="str">
-        <x:v>WINBACK_2025_06</x:v>
+        <x:v>1-5</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="13" t="str">
-        <x:v>marketing_experiment.csv</x:v>
+        <x:v>rides.csv</x:v>
       </x:c>
       <x:c r="B53" s="13" t="str">
-        <x:v>customer_id</x:v>
+        <x:v>vehicle_quality</x:v>
       </x:c>
       <x:c r="C53" s="13" t="str">
         <x:v>character</x:v>
       </x:c>
       <x:c r="D53" s="13" t="str">
-        <x:v>Randomized customer identifier</x:v>
+        <x:v>MetroRide vehicle category</x:v>
       </x:c>
       <x:c r="E53" s="13" t="str">
-        <x:v>Joins to customers.csv</x:v>
+        <x:v>Standard; Comfort; Premium</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="13" t="str">
-        <x:v>marketing_experiment.csv</x:v>
+        <x:v>rides.csv</x:v>
       </x:c>
       <x:c r="B54" s="13" t="str">
-        <x:v>assignment_date</x:v>
+        <x:v>customer_rating</x:v>
       </x:c>
       <x:c r="C54" s="13" t="str">
-        <x:v>date</x:v>
+        <x:v>integer</x:v>
       </x:c>
       <x:c r="D54" s="13" t="str">
-        <x:v>Campaign assignment date</x:v>
+        <x:v>Rating submitted after completed ride</x:v>
       </x:c>
       <x:c r="E54" s="13" t="str">
-        <x:v>YYYY-MM-DD</x:v>
+        <x:v>1-5; blank if no rating</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="13" t="str">
-        <x:v>marketing_experiment.csv</x:v>
+        <x:v>rides.csv</x:v>
       </x:c>
       <x:c r="B55" s="13" t="str">
-        <x:v>treatment_group</x:v>
+        <x:v>complaint</x:v>
       </x:c>
       <x:c r="C55" s="13" t="str">
-        <x:v>character</x:v>
+        <x:v>integer</x:v>
       </x:c>
       <x:c r="D55" s="13" t="str">
-        <x:v>Randomly assigned campaign condition</x:v>
+        <x:v>Whether customer filed a complaint about request</x:v>
       </x:c>
       <x:c r="E55" s="13" t="str">
-        <x:v>Five conditions including Control</x:v>
+        <x:v>1=yes; 0=no</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -1258,16 +1258,16 @@
         <x:v>marketing_experiment.csv</x:v>
       </x:c>
       <x:c r="B56" s="13" t="str">
-        <x:v>offer_value</x:v>
+        <x:v>campaign_id</x:v>
       </x:c>
       <x:c r="C56" s="13" t="str">
-        <x:v>double</x:v>
+        <x:v>character</x:v>
       </x:c>
       <x:c r="D56" s="13" t="str">
-        <x:v>Nominal value associated with assigned offer</x:v>
+        <x:v>Campaign identifier</x:v>
       </x:c>
       <x:c r="E56" s="13" t="str">
-        <x:v>USD; percentage offer uses expected nominal value</x:v>
+        <x:v>WINBACK_2025_06</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
@@ -1275,16 +1275,16 @@
         <x:v>marketing_experiment.csv</x:v>
       </x:c>
       <x:c r="B57" s="13" t="str">
-        <x:v>message_type</x:v>
+        <x:v>customer_id</x:v>
       </x:c>
       <x:c r="C57" s="13" t="str">
         <x:v>character</x:v>
       </x:c>
       <x:c r="D57" s="13" t="str">
-        <x:v>Marketing message emphasis</x:v>
+        <x:v>Randomized customer identifier</x:v>
       </x:c>
       <x:c r="E57" s="13" t="str">
-        <x:v>No message for control</x:v>
+        <x:v>Joins to customers.csv</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
@@ -1292,16 +1292,16 @@
         <x:v>marketing_experiment.csv</x:v>
       </x:c>
       <x:c r="B58" s="13" t="str">
-        <x:v>offer_opened</x:v>
+        <x:v>assignment_date</x:v>
       </x:c>
       <x:c r="C58" s="13" t="str">
-        <x:v>integer</x:v>
+        <x:v>date</x:v>
       </x:c>
       <x:c r="D58" s="13" t="str">
-        <x:v>Whether customer opened campaign message</x:v>
+        <x:v>Campaign assignment date</x:v>
       </x:c>
       <x:c r="E58" s="13" t="str">
-        <x:v>1=yes; 0=no</x:v>
+        <x:v>YYYY-MM-DD</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
@@ -1309,16 +1309,16 @@
         <x:v>marketing_experiment.csv</x:v>
       </x:c>
       <x:c r="B59" s="13" t="str">
-        <x:v>booked_within_30d</x:v>
+        <x:v>treatment_group</x:v>
       </x:c>
       <x:c r="C59" s="13" t="str">
-        <x:v>integer</x:v>
+        <x:v>character</x:v>
       </x:c>
       <x:c r="D59" s="13" t="str">
-        <x:v>Whether customer booked within 30 days after assignment</x:v>
+        <x:v>Randomly assigned campaign condition</x:v>
       </x:c>
       <x:c r="E59" s="13" t="str">
-        <x:v>1=yes; 0=no</x:v>
+        <x:v>Five conditions including Control</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
@@ -1326,16 +1326,16 @@
         <x:v>marketing_experiment.csv</x:v>
       </x:c>
       <x:c r="B60" s="13" t="str">
-        <x:v>rides_within_30d</x:v>
+        <x:v>offer_amount</x:v>
       </x:c>
       <x:c r="C60" s="13" t="str">
-        <x:v>integer</x:v>
+        <x:v>double</x:v>
       </x:c>
       <x:c r="D60" s="13" t="str">
-        <x:v>Rides booked within 30-day follow-up window</x:v>
+        <x:v>Dollar amount associated with assigned offer</x:v>
       </x:c>
       <x:c r="E60" s="13" t="str">
-        <x:v>Count</x:v>
+        <x:v>USD; zero for control; message only; and percentage offer</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
@@ -1343,16 +1343,16 @@
         <x:v>marketing_experiment.csv</x:v>
       </x:c>
       <x:c r="B61" s="13" t="str">
-        <x:v>gross_spend_within_30d</x:v>
+        <x:v>offer_percent</x:v>
       </x:c>
       <x:c r="C61" s="13" t="str">
         <x:v>double</x:v>
       </x:c>
       <x:c r="D61" s="13" t="str">
-        <x:v>Gross customer spending during follow-up</x:v>
+        <x:v>Percentage discount associated with assigned offer</x:v>
       </x:c>
       <x:c r="E61" s="13" t="str">
-        <x:v>USD</x:v>
+        <x:v>Decimal; 0.20 for 20% off and zero otherwise</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
@@ -1360,16 +1360,16 @@
         <x:v>marketing_experiment.csv</x:v>
       </x:c>
       <x:c r="B62" s="13" t="str">
-        <x:v>offer_redeemed</x:v>
+        <x:v>message_type</x:v>
       </x:c>
       <x:c r="C62" s="13" t="str">
-        <x:v>integer</x:v>
+        <x:v>character</x:v>
       </x:c>
       <x:c r="D62" s="13" t="str">
-        <x:v>Whether assigned financial offer was redeemed</x:v>
+        <x:v>Marketing message emphasis</x:v>
       </x:c>
       <x:c r="E62" s="13" t="str">
-        <x:v>1=yes; 0=no</x:v>
+        <x:v>No message for control</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
@@ -1377,16 +1377,16 @@
         <x:v>marketing_experiment.csv</x:v>
       </x:c>
       <x:c r="B63" s="13" t="str">
-        <x:v>promotion_cost</x:v>
+        <x:v>offer_opened</x:v>
       </x:c>
       <x:c r="C63" s="13" t="str">
-        <x:v>double</x:v>
+        <x:v>integer</x:v>
       </x:c>
       <x:c r="D63" s="13" t="str">
-        <x:v>Promotion cost incurred by MetroRide</x:v>
+        <x:v>Whether customer opened campaign message</x:v>
       </x:c>
       <x:c r="E63" s="13" t="str">
-        <x:v>USD</x:v>
+        <x:v>1=yes; 0=no</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
@@ -1394,32 +1394,117 @@
         <x:v>marketing_experiment.csv</x:v>
       </x:c>
       <x:c r="B64" s="13" t="str">
+        <x:v>booked_within_30d</x:v>
+      </x:c>
+      <x:c r="C64" s="13" t="str">
+        <x:v>integer</x:v>
+      </x:c>
+      <x:c r="D64" s="13" t="str">
+        <x:v>Whether customer requested at least one ride within 30 days after assignment</x:v>
+      </x:c>
+      <x:c r="E64" s="13" t="str">
+        <x:v>1=yes; 0=no</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" s="13" t="str">
+        <x:v>marketing_experiment.csv</x:v>
+      </x:c>
+      <x:c r="B65" s="13" t="str">
+        <x:v>rides_within_30d</x:v>
+      </x:c>
+      <x:c r="C65" s="13" t="str">
+        <x:v>integer</x:v>
+      </x:c>
+      <x:c r="D65" s="13" t="str">
+        <x:v>Completed rides within the 30-day follow-up window</x:v>
+      </x:c>
+      <x:c r="E65" s="13" t="str">
+        <x:v>Count</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" s="13" t="str">
+        <x:v>marketing_experiment.csv</x:v>
+      </x:c>
+      <x:c r="B66" s="13" t="str">
+        <x:v>gross_spend_within_30d</x:v>
+      </x:c>
+      <x:c r="C66" s="13" t="str">
+        <x:v>double</x:v>
+      </x:c>
+      <x:c r="D66" s="13" t="str">
+        <x:v>Fares and Priority fees before campaign discounts during follow-up</x:v>
+      </x:c>
+      <x:c r="E66" s="13" t="str">
+        <x:v>USD; completed rides only</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" s="13" t="str">
+        <x:v>marketing_experiment.csv</x:v>
+      </x:c>
+      <x:c r="B67" s="13" t="str">
+        <x:v>offer_redeemed</x:v>
+      </x:c>
+      <x:c r="C67" s="13" t="str">
+        <x:v>integer</x:v>
+      </x:c>
+      <x:c r="D67" s="13" t="str">
+        <x:v>Whether assigned financial offer was redeemed</x:v>
+      </x:c>
+      <x:c r="E67" s="13" t="str">
+        <x:v>1=yes; 0=no</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" s="13" t="str">
+        <x:v>marketing_experiment.csv</x:v>
+      </x:c>
+      <x:c r="B68" s="13" t="str">
+        <x:v>promotion_cost</x:v>
+      </x:c>
+      <x:c r="C68" s="13" t="str">
+        <x:v>double</x:v>
+      </x:c>
+      <x:c r="D68" s="13" t="str">
+        <x:v>Campaign discount or ride credit incurred by MetroRide</x:v>
+      </x:c>
+      <x:c r="E68" s="13" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" s="13" t="str">
+        <x:v>marketing_experiment.csv</x:v>
+      </x:c>
+      <x:c r="B69" s="13" t="str">
         <x:v>net_revenue_within_30d</x:v>
       </x:c>
-      <x:c r="C64" s="13" t="str">
-        <x:v>double</x:v>
-      </x:c>
-      <x:c r="D64" s="13" t="str">
-        <x:v>MetroRide revenue share less promotion cost</x:v>
-      </x:c>
-      <x:c r="E64" s="13" t="str">
+      <x:c r="C69" s="13" t="str">
+        <x:v>double</x:v>
+      </x:c>
+      <x:c r="D69" s="13" t="str">
+        <x:v>72% of gross spend less campaign promotion cost</x:v>
+      </x:c>
+      <x:c r="E69" s="13" t="str">
         <x:v>USD</x:v>
       </x:c>
     </x:row>
-    <x:row r="65">
-      <x:c r="A65" s="14" t="str">
+    <x:row r="70">
+      <x:c r="A70" s="14" t="str">
         <x:v>marketing_experiment.csv</x:v>
       </x:c>
-      <x:c r="B65" s="14" t="str">
+      <x:c r="B70" s="14" t="str">
         <x:v>retained_within_60d</x:v>
       </x:c>
-      <x:c r="C65" s="14" t="str">
-        <x:v>integer</x:v>
-      </x:c>
-      <x:c r="D65" s="14" t="str">
-        <x:v>Whether customer used MetroRide in the subsequent retention window</x:v>
-      </x:c>
-      <x:c r="E65" s="14" t="str">
+      <x:c r="C70" s="14" t="str">
+        <x:v>integer</x:v>
+      </x:c>
+      <x:c r="D70" s="14" t="str">
+        <x:v>Whether customer completed a ride during days 31-60 after assignment</x:v>
+      </x:c>
+      <x:c r="E70" s="14" t="str">
         <x:v>1=yes; 0=no</x:v>
       </x:c>
     </x:row>

</xml_diff>